<commit_message>
Statistics on the number of days the CSI 1000 Index triggered 5% and 10% fluctuations
</commit_message>
<xml_diff>
--- a/stock1.xlsx
+++ b/stock1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubZhuyanxi\CarnoFinance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41879F7-CCEE-48EE-9E45-6107E3633738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4886A6-2E61-47EF-9F78-34A695EC170C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FF009721-C680-46B5-A86A-A7B389958F06}"/>
+    <workbookView xWindow="12555" yWindow="3075" windowWidth="20220" windowHeight="10770" xr2:uid="{FF009721-C680-46B5-A86A-A7B389958F06}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -455,7 +455,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -475,18 +475,18 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>100</v>
+        <v>93.22</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
         <f>C2+A3*(B3-B2)</f>
-        <v>100</v>
+        <v>93.22</v>
       </c>
       <c r="D3">
         <f>C3/B3</f>
-        <v>100</v>
+        <v>93.22</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -498,176 +498,176 @@
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>A3*(1-A2)</f>
-        <v>80</v>
+        <v>79.236999999999995</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4">
         <f>C3+A4*(B4-B3)</f>
-        <v>260</v>
+        <v>251.69399999999999</v>
       </c>
       <c r="D4">
         <f>C4/B4</f>
-        <v>86.666666666666671</v>
+        <v>83.897999999999996</v>
       </c>
       <c r="E4">
         <f>(A4/D3-1)*100</f>
-        <v>-19.999999999999996</v>
+        <v>-15.000000000000002</v>
       </c>
       <c r="F4">
         <f>(A4/D4-1)*100</f>
-        <v>-7.6923076923076987</v>
+        <v>-5.555555555555558</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <f>A3*(1-A2*2)</f>
-        <v>60</v>
+        <v>65.253999999999991</v>
       </c>
       <c r="B5">
         <v>6</v>
       </c>
       <c r="C5">
         <f>C4+A5*(B5-B4)</f>
-        <v>440</v>
+        <v>447.45599999999996</v>
       </c>
       <c r="D5">
         <f>C5/B5</f>
-        <v>73.333333333333329</v>
+        <v>74.575999999999993</v>
       </c>
       <c r="E5">
         <f t="shared" ref="E5:E10" si="0">(A5/D4-1)*100</f>
-        <v>-30.76923076923077</v>
+        <v>-22.222222222222232</v>
       </c>
       <c r="F5">
         <f t="shared" ref="F5:F10" si="1">(A5/D5-1)*100</f>
-        <v>-18.181818181818176</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <f>A3*(1-A2*3)</f>
-        <v>39.999999999999993</v>
+        <v>51.271000000000001</v>
       </c>
       <c r="B6">
         <v>10</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="2">C5+A6*(B6-B5)</f>
-        <v>600</v>
+        <v>652.54</v>
       </c>
       <c r="D6">
         <f t="shared" ref="D6:D10" si="3">C6/B6</f>
-        <v>60</v>
+        <v>65.253999999999991</v>
       </c>
       <c r="E6">
         <f t="shared" si="0"/>
-        <v>-45.45454545454546</v>
+        <v>-31.249999999999989</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>-33.33333333333335</v>
+        <v>-21.42857142857142</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <f>A3*(1-A2*4)</f>
-        <v>19.999999999999996</v>
+        <v>37.288000000000004</v>
       </c>
       <c r="B7">
         <v>15</v>
       </c>
       <c r="C7">
         <f t="shared" si="2"/>
-        <v>700</v>
+        <v>838.98</v>
       </c>
       <c r="D7">
         <f t="shared" si="3"/>
-        <v>46.666666666666664</v>
+        <v>55.932000000000002</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>-66.666666666666671</v>
+        <v>-42.85714285714284</v>
       </c>
       <c r="F7">
         <f t="shared" si="1"/>
-        <v>-57.142857142857153</v>
+        <v>-33.333333333333329</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <f>A3*(1-A2*5)</f>
-        <v>0</v>
+        <v>23.305</v>
       </c>
       <c r="B8">
         <v>21</v>
       </c>
       <c r="C8">
         <f t="shared" si="2"/>
-        <v>700</v>
+        <v>978.81</v>
       </c>
       <c r="D8">
         <f t="shared" si="3"/>
-        <v>33.333333333333336</v>
+        <v>46.61</v>
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>-100</v>
+        <v>-58.333333333333336</v>
       </c>
       <c r="F8">
         <f t="shared" si="1"/>
-        <v>-100</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <f>A3*(1-A2*6)</f>
-        <v>-20.000000000000018</v>
+        <v>9.3220000000000081</v>
       </c>
       <c r="B9">
         <v>28</v>
       </c>
       <c r="C9">
         <f t="shared" si="2"/>
-        <v>559.99999999999989</v>
+        <v>1044.0640000000001</v>
       </c>
       <c r="D9">
         <f t="shared" si="3"/>
-        <v>19.999999999999996</v>
+        <v>37.288000000000004</v>
       </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>-160.00000000000006</v>
+        <v>-79.999999999999986</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>-200.00000000000009</v>
+        <v>-74.999999999999972</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <f>A3*(1-A2*7)</f>
-        <v>-40.000000000000014</v>
+        <v>-4.661000000000004</v>
       </c>
       <c r="B10">
         <v>36</v>
       </c>
       <c r="C10">
         <f t="shared" si="2"/>
-        <v>239.99999999999977</v>
+        <v>1006.7760000000001</v>
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>6.6666666666666607</v>
+        <v>27.966000000000001</v>
       </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>-300.00000000000011</v>
+        <v>-112.5</v>
       </c>
       <c r="F10">
         <f t="shared" si="1"/>
-        <v>-700.00000000000068</v>
+        <v>-116.66666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>